<commit_message>
added sketches and assignment 1 taskes 5-7
</commit_message>
<xml_diff>
--- a/passenger-data.xlsx
+++ b/passenger-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\cs424-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9760970A-2808-4749-8E4A-0898F1822CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3410D41-771A-4FE5-8790-F0CC56D95BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{2FAE1D98-6047-4A29-AB5F-53D26DEB9837}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{2FAE1D98-6047-4A29-AB5F-53D26DEB9837}"/>
   </bookViews>
   <sheets>
     <sheet name="Inbound" sheetId="1" r:id="rId1"/>

</xml_diff>